<commit_message>
fix: eventos usan nombre canónico del país en lugar de ISO code
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eventos_prueba.xlsx
+++ b/eventos_prueba.xlsx
@@ -439,7 +439,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>pais_iso</t>
+          <t>pais</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -469,7 +469,6 @@
           <t>global</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>#ef5350</t>
@@ -497,7 +496,6 @@
           <t>global</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>#ef5350</t>
@@ -525,7 +523,6 @@
           <t>global</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>#ef5350</t>
@@ -553,7 +550,6 @@
           <t>global</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>#ff9800</t>
@@ -581,7 +577,6 @@
           <t>global</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>#ef5350</t>
@@ -609,7 +604,6 @@
           <t>global</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>#ff9800</t>
@@ -637,7 +631,6 @@
           <t>global</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>#ff9800</t>
@@ -665,7 +658,6 @@
           <t>global</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>#ff9800</t>
@@ -693,7 +685,6 @@
           <t>global</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>#ff9800</t>
@@ -721,7 +712,6 @@
           <t>global</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>#ef5350</t>
@@ -749,7 +739,6 @@
           <t>global</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>#ff9800</t>
@@ -777,7 +766,6 @@
           <t>global</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>#ef5350</t>
@@ -805,7 +793,6 @@
           <t>global</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>#ff9800</t>
@@ -835,7 +822,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -867,7 +854,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -899,7 +886,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -931,7 +918,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -963,7 +950,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -995,7 +982,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1027,7 +1014,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1059,7 +1046,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1091,7 +1078,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1123,7 +1110,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1155,7 +1142,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1187,7 +1174,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1219,7 +1206,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1251,7 +1238,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1283,7 +1270,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1315,7 +1302,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1347,7 +1334,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1379,7 +1366,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1411,7 +1398,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1443,7 +1430,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1475,7 +1462,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1507,7 +1494,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1539,7 +1526,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1571,7 +1558,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1603,7 +1590,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1635,7 +1622,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1667,7 +1654,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1699,7 +1686,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1731,7 +1718,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -1763,7 +1750,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">

</xml_diff>

<commit_message>
feat: ampliar eventos_prueba.xlsx de 43 a 79 eventos
Nuevos eventos por región:
- Global: Brexit referéndum, boom IA
- USA: Obama 2008/2012, QE2, debt ceiling 2011/2023, Tax Reform, CARES Act
- Argentina: Hiperinflación, Convertibilidad, YPF expropiación, Griesa, elecciones 2015, regreso mercados
- Brasil: Lava Jato, impeachment Dilma, Bolsonaro, Lula, 8 enero 2023
- México: AMLO, T-MEC, Sheinbaum
- Europa: Draghi, crisis Grecia, Brexit efectivo, crisis energética
- China: OMC, Wuhan lockdown, regulación tech, fin cero COVID

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eventos_prueba.xlsx
+++ b/eventos_prueba.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1759,6 +1759,1143 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Brexit — referéndum UK</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2016-06-23</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2016-06-24</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>#ef5350</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Pandemia COVID — inicio cuarentenas</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2020-03-11</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2020-04-30</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>#ef5350</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Boom inteligencia artificial</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2022-11-30</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>#4caf50</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Elecciones USA 2008 — Obama</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2008-11-04</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2008-11-04</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>#2196f3</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Cuantitative Easing QE2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2010-11-03</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2011-06-30</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>#2196f3</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Crisis techo de deuda USA</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2011-07-22</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2011-08-09</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>#ff9800</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Elecciones USA 2012 — Obama</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2012-11-06</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2012-11-06</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>#2196f3</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Reforma fiscal Trump — Tax Cuts</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2017-12-22</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2017-12-22</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>#4caf50</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>CARES Act — estímulo COVID</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2020-03-27</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2020-03-27</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>#4caf50</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Techo deuda USA 2023</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2023-01-19</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2023-06-03</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>#ff9800</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Hiperinflación argentina</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1989-01-01</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>1991-03-31</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>#ef5350</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Plan de Convertibilidad</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1991-04-01</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2001-11-30</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>#4caf50</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Expropiación YPF</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2012-04-16</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2012-05-03</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>#ff9800</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Fallo fondos buitre — Griesa</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2014-07-30</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2016-04-22</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>#ef5350</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>PASO 2015 — Macri vs Scioli</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2015-08-09</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2015-08-09</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>#2196f3</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Elecciones presidenciales 2015</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2015-11-22</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2015-11-22</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>#2196f3</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Regreso a mercados internacionales</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2016-04-19</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2016-04-22</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>#4caf50</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Elecciones PASO 2017 — Cristina</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2017-10-22</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>2017-10-22</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>#2196f3</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Acuerdo con bonistas — fin default</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2016-02-29</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>2016-04-22</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>#4caf50</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Operación Lava Jato</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2014-03-17</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>2021-02-08</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>#ff9800</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Impeachment Dilma Rousseff</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2016-04-17</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>2016-08-31</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>#ef5350</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Elecciones Brasil 2018 — Bolsonaro</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2018-10-28</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>2018-10-28</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>#2196f3</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>COVID — impacto Brasil</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2020-03-11</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2021-12-31</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>#ef5350</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Elecciones Brasil 2022 — Lula</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2022-10-30</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2022-10-30</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>#2196f3</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Intento de golpe — 8 enero 2023</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2023-01-08</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2023-01-08</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>#ef5350</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Elecciones México 2018 — AMLO</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2018-07-01</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2018-07-01</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>#2196f3</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>T-MEC / USMCA entra en vigor</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2020-07-01</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2020-07-01</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>#4caf50</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Elecciones México 2024 — Sheinbaum</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2024-06-02</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2024-06-02</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>#2196f3</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Crisis Grecia — riesgo Grexit</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2015-06-26</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2015-07-13</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>#ef5350</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Draghi — whatever it takes</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2012-07-26</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2012-07-26</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>#4caf50</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Brexit efectivo — UK sale de la UE</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2020-01-31</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>2020-01-31</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>#ff9800</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Crisis energética Europa</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2021-09-01</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>2023-03-31</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>#ff9800</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>China ingresa a la OMC</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2001-12-11</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>2001-12-11</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>#4caf50</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Lockdown COVID — Wuhan</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2020-01-23</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>2020-04-08</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>#ef5350</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Regulación sector tech chino</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>2022-12-31</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>#ef5350</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Fin política cero COVID — China</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2022-12-07</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>2022-12-31</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>#4caf50</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>